<commit_message>
Atualizacao adicionar linhas ignoradas
</commit_message>
<xml_diff>
--- a/Comparação de Encerrantes.xlsx
+++ b/Comparação de Encerrantes.xlsx
@@ -10,25 +10,25 @@
     <sheet name="Page 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Page 1'!$A$1:$F$25</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Page 1'!$A$1:$F$29</definedName>
   </definedNames>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="32">
   <si>
     <t>Comparação de Encerrantes</t>
   </si>
   <si>
-    <t>Data do Movimento: 27/07/2026</t>
-  </si>
-  <si>
-    <t>28/07/2026 16:07:01</t>
-  </si>
-  <si>
-    <t>Empresa: POSTO CABRAL 5</t>
+    <t>Data do Movimento: 19/08/2026</t>
+  </si>
+  <si>
+    <t>20/08/2026 08:08:11</t>
+  </si>
+  <si>
+    <t>Empresa: REDE ED+ IPANEMA LTDA</t>
   </si>
   <si>
     <t>Bico</t>
@@ -46,36 +46,36 @@
     <t>1</t>
   </si>
   <si>
-    <t>DIESEL S-500</t>
+    <t>OLEO DIESEL B S10 - COMUM</t>
   </si>
   <si>
     <t>2</t>
   </si>
   <si>
+    <t>OLEO DIESEL S500</t>
+  </si>
+  <si>
     <t>3</t>
   </si>
   <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>ETANOL COMUM</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
     <t>GASOLINA COMUM</t>
   </si>
   <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>ETANOL COMUM</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
     <t>7</t>
   </si>
   <si>
-    <t>DIESEL S-10</t>
-  </si>
-  <si>
     <t>8</t>
   </si>
   <si>
@@ -91,13 +91,25 @@
     <t>12</t>
   </si>
   <si>
-    <t>Total da Diferença da Empresa POSTO CABRAL 5</t>
+    <t>13</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>Total da Diferença da Empresa REDE ED+ IPANEMA LTDA</t>
   </si>
   <si>
     <t>Total Geral</t>
   </si>
   <si>
-    <t>Adaptive Business 3.26.01.46 r1063 p875 - Gestão Inteligente de Negócios. (T.E.= 1,007s)</t>
+    <t>Adaptive Business 3.26.01.46 r1063 p875 - Gestão Inteligente de Negócios. (T.E.= 0,48s)</t>
   </si>
   <si>
     <t>Página: 1 de 1</t>
@@ -294,7 +306,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.09953194944" customWidth="1"/>
@@ -362,14 +374,14 @@
         <v>9</v>
       </c>
       <c r="C6" s="8">
-        <v>795499.71</v>
+        <v>584784.95</v>
       </c>
       <c r="D6" s="8">
-        <v>32.15</v>
+        <v>584784.023</v>
       </c>
       <c r="E6" s="8"/>
       <c r="F6" s="8">
-        <v>795467.56</v>
+        <v>0.927</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="11.6352" customHeight="1">
@@ -377,35 +389,35 @@
         <v>10</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C7" s="10">
-        <v>807553.33</v>
+        <v>518816.52</v>
       </c>
       <c r="D7" s="10">
-        <v>0.11</v>
+        <v>518816.285</v>
       </c>
       <c r="E7" s="10"/>
       <c r="F7" s="10">
-        <v>807553.22</v>
+        <v>0.235</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="11.6352" customHeight="1">
       <c r="A8" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="7" t="s">
-        <v>12</v>
-      </c>
       <c r="C8" s="8">
-        <v>596386.15</v>
+        <v>271576.2</v>
       </c>
       <c r="D8" s="8">
-        <v>20.08</v>
+        <v>271576.065</v>
       </c>
       <c r="E8" s="8"/>
       <c r="F8" s="8">
-        <v>596366.07</v>
+        <v>0.135</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="11.6352" customHeight="1">
@@ -413,17 +425,17 @@
         <v>13</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C9" s="10">
-        <v>716778.86</v>
+        <v>539962.76</v>
       </c>
       <c r="D9" s="10">
-        <v>20.07</v>
+        <v>539962.556</v>
       </c>
       <c r="E9" s="10"/>
       <c r="F9" s="10">
-        <v>716758.79</v>
+        <v>0.204</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="10.908" customHeight="1">
@@ -434,14 +446,14 @@
         <v>15</v>
       </c>
       <c r="C10" s="8">
-        <v>0</v>
+        <v>1266042.35</v>
       </c>
       <c r="D10" s="8">
-        <v>0</v>
+        <v>1266051.244</v>
       </c>
       <c r="E10" s="8"/>
       <c r="F10" s="8">
-        <v>0</v>
+        <v>-8.894</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="11.6352" customHeight="1">
@@ -449,35 +461,35 @@
         <v>16</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C11" s="10">
-        <v>716791.45</v>
+        <v>898245.12</v>
       </c>
       <c r="D11" s="10">
-        <v>12.53</v>
+        <v>898251.748</v>
       </c>
       <c r="E11" s="10"/>
       <c r="F11" s="10">
-        <v>716778.92</v>
+        <v>-6.628</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="11.6352" customHeight="1">
       <c r="A12" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="7" t="s">
-        <v>18</v>
-      </c>
       <c r="C12" s="8">
-        <v>1979071.08</v>
+        <v>323236.02</v>
       </c>
       <c r="D12" s="8">
-        <v>95.78</v>
+        <v>323235.297</v>
       </c>
       <c r="E12" s="8"/>
       <c r="F12" s="8">
-        <v>1978975.3</v>
+        <v>0.723</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="11.6352" customHeight="1">
@@ -485,17 +497,17 @@
         <v>19</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C13" s="10">
-        <v>1354331.31</v>
+        <v>747427.61</v>
       </c>
       <c r="D13" s="10">
-        <v>21.49</v>
+        <v>747425.775</v>
       </c>
       <c r="E13" s="10"/>
       <c r="F13" s="10">
-        <v>1354309.82</v>
+        <v>1.835</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="10.908" customHeight="1">
@@ -503,17 +515,17 @@
         <v>20</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C14" s="8">
-        <v>1345904.72</v>
+        <v>297141.37</v>
       </c>
       <c r="D14" s="8">
-        <v>73.082</v>
+        <v>297144.853</v>
       </c>
       <c r="E14" s="8"/>
       <c r="F14" s="8">
-        <v>1345831.638</v>
+        <v>-3.483</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="11.6352" customHeight="1">
@@ -521,17 +533,17 @@
         <v>21</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C15" s="10">
-        <v>1026765.12</v>
+        <v>896409</v>
       </c>
       <c r="D15" s="10">
-        <v>59.74</v>
+        <v>896370.138</v>
       </c>
       <c r="E15" s="10"/>
       <c r="F15" s="10">
-        <v>1026705.38</v>
+        <v>38.862</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="11.6352" customHeight="1">
@@ -542,14 +554,14 @@
         <v>15</v>
       </c>
       <c r="C16" s="8">
-        <v>2044047.18</v>
+        <v>957615.33</v>
       </c>
       <c r="D16" s="8">
-        <v>38.35</v>
+        <v>957614.541</v>
       </c>
       <c r="E16" s="8"/>
       <c r="F16" s="8">
-        <v>2044008.83</v>
+        <v>0.789</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="11.6352" customHeight="1">
@@ -557,69 +569,141 @@
         <v>23</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C17" s="10">
-        <v>1418124.86</v>
+        <v>1354132.83</v>
       </c>
       <c r="D17" s="10">
-        <v>11.47</v>
+        <v>1354136.652</v>
       </c>
       <c r="E17" s="10"/>
       <c r="F17" s="10">
-        <v>1418113.39</v>
+        <v>-3.822</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="10.908" customHeight="1">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="12">
-        <v>12800868.918</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="5.8176" customHeight="1"/>
+      <c r="B18" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C18" s="8">
+        <v>494696.91</v>
+      </c>
+      <c r="D18" s="8">
+        <v>494695.192</v>
+      </c>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8">
+        <v>1.718</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="11.6352" customHeight="1">
+      <c r="A19" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19" s="10">
+        <v>171934.24</v>
+      </c>
+      <c r="D19" s="10">
+        <v>171934.092</v>
+      </c>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10">
+        <v>0.148</v>
+      </c>
+    </row>
     <row r="20" spans="1:6" ht="11.6352" customHeight="1">
-      <c r="A20" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="14">
-        <v>12800868.918</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="145.44" customHeight="1"/>
-    <row r="22" spans="1:6" ht="145.44" customHeight="1"/>
-    <row r="23" spans="1:6" ht="130.896" customHeight="1"/>
-    <row r="24" spans="1:6" ht="130.896" customHeight="1">
-      <c r="A24" s="15"/>
-      <c r="B24" s="15"/>
-      <c r="C24" s="15"/>
-      <c r="D24" s="15"/>
-      <c r="E24" s="15"/>
-      <c r="F24" s="15"/>
-    </row>
-    <row r="25" spans="1:6" ht="11.6352" customHeight="1">
-      <c r="A25" s="16" t="s">
+      <c r="A20" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="16"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="17" t="s">
+      <c r="B20" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C20" s="8">
+        <v>792867.23</v>
+      </c>
+      <c r="D20" s="8">
+        <v>792860.437</v>
+      </c>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8">
+        <v>6.793</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="11.6352" customHeight="1">
+      <c r="A21" s="5" t="s">
         <v>27</v>
       </c>
+      <c r="B21" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="10">
+        <v>702963.06</v>
+      </c>
+      <c r="D21" s="10">
+        <v>702961.06</v>
+      </c>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="10.908" customHeight="1">
+      <c r="A22" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="12">
+        <v>31.542</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="5.8176" customHeight="1"/>
+    <row r="24" spans="1:6" ht="11.6352" customHeight="1">
+      <c r="A24" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="14">
+        <v>31.542</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="145.44" customHeight="1"/>
+    <row r="26" spans="1:6" ht="145.44" customHeight="1"/>
+    <row r="27" spans="1:6" ht="108.35279999999999" customHeight="1"/>
+    <row r="28" spans="1:6" ht="107.62559999999999" customHeight="1">
+      <c r="A28" s="15"/>
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+    </row>
+    <row r="29" spans="1:6" ht="11.6352" customHeight="1">
+      <c r="A29" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" s="16"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="17" t="s">
+        <v>31</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="25">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="E2:F2"/>
@@ -638,9 +722,13 @@
     <mergeCell ref="D15:E15"/>
     <mergeCell ref="D16:E16"/>
     <mergeCell ref="D17:E17"/>
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A29:E29"/>
   </mergeCells>
   <pageMargins left="0.3937007874015748" right="0.3937007874015748" top="0.3937007874015748" bottom="0.3937007874015748" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" fitToHeight="0"/>

</xml_diff>